<commit_message>
Vectorización del mazo y reducción de dimensionalidad
</commit_message>
<xml_diff>
--- a/lor_dataset.xlsx
+++ b/lor_dataset.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1268,16 +1268,20 @@
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
-        <v>14</v>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Evilkyatt</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
-        <v>130</v>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>130.0</t>
+        </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -1294,11 +1298,15 @@
           <t>Bilgewater|Demacia|Freljord|Mount Targon|Piltover &amp; Zaun|Shadow Isles</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>16</v>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
@@ -1316,16 +1324,20 @@
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
-        <v>19</v>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Im Bard Out</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
-        <v>101</v>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>101.0</t>
+        </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -1342,11 +1354,15 @@
           <t>Bandle City|F18|Freljord|Mount Targon|Shurima</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>17</v>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
@@ -1364,16 +1380,20 @@
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
-        <v>29</v>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Carrot Spirit</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
-        <v>100</v>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -1390,11 +1410,15 @@
           <t>Bandle City|Noxus</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I17" s="2" t="n">
-        <v>14</v>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
@@ -1406,6 +1430,592 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>mbrookz</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>124.0</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>iMQDykjthqoztGrFSrHwtphL2pV9BIrGgAz1EIFDSRHTboYbSYy9SPFPyLCvPzq3i5PdNMVJIeWEiA</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>CIEQCAIADUAQEAAGAECAAAYBAUAAYAIGAYOQCBQEBAAQOAAFAEEAABQEAYAAMCQVDQBACAIABIAQMABAAA</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Bilgewater|Demacia|Piltover &amp; Zaun</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01DE029","n":3},{"c":"02DE006","n":3},{"c":"04DE003","n":3},{"c":"05DE012","n":3},{"c":"06BW029","n":3},{"c":"06PZ008","n":3},{"c":"07DE005","n":3},{"c":"08DE006","n":3},{"c":"06DE006","n":3},{"c":"06DE010","n":3},{"c":"06DE021","n":3},{"c":"06DE028","n":3},{"c":"01DE010","n":2},{"c":"06DE032","n":2}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>NotreDammit</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ik2qUvSnwi86IeXEu5fiNj4mTgE6LR2fHlKi_J1gS05olorTm2il2QpyaTh-gdM17lDLdfXLjcZ3lw</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>CQDACBQKDIAQQCQFAEEAIGACA4FASFADAECAQGJUAMCQIAQGBYBQCAIEGUAQEBAKAECQURQBAEDAIKY</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|Bilgewater|Piltover &amp; Zaun</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"06BC026","n":3},{"c":"08BC005","n":3},{"c":"08PZ024","n":3},{"c":"07BC009","n":3},{"c":"07BC020","n":3},{"c":"01PZ008","n":3},{"c":"01PZ025","n":3},{"c":"01PZ052","n":3},{"c":"05PZ002","n":3},{"c":"05PZ006","n":3},{"c":"05PZ014","n":3},{"c":"01PZ053","n":2},{"c":"02PZ010","n":2},{"c":"05BC070","n":2},{"c":"01BW004","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Scilla</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>vwIBeem3KeMHt2DXT689hGEUoZwydZ1S7q2GcWLHvl4GxNDmaxHhI4X25Rx9afLQ0Z4io5Xm3dC2-A</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>CEAAAAICAAAAMJY</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Demacia</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"02DE000","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>netinho99</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>pv-ejnBJpvr2-uknjMz4mPMiw3R4DenY9PoZl1KIB13JDHHA0bveLZ52rxlSXCMHyWvTBN-0c4ubjw</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>CMCQCBADB4AQOBZHAIDAOBAFAMAQGEY2EYBQIBYFCQ3QIAIBAMFQCAYDAMAQIAYKAECAOOYCAECAGFQBBADQE</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Freljord|Noxus|Piltover &amp; Zaun|Shurima</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04NX015","n":3},{"c":"07SH039","n":3},{"c":"06SH004","n":3},{"c":"06SH005","n":3},{"c":"01NX019","n":3},{"c":"01NX026","n":3},{"c":"01NX038","n":3},{"c":"04SH005","n":3},{"c":"04SH020","n":3},{"c":"04SH055","n":3},{"c":"01NX011","n":2},{"c":"03NX003","n":2},{"c":"04NX010","n":2},{"c":"04SH059","n":2},{"c":"01PZ003","n":1},{"c":"22FR008","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ANG3L</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>64T_QJuxrjgymcgVU_WRi83XMzxl5n3CFbhCLnEpra1r8axDA_rRCCP2Lvk2rIRx-TL7jn-FAfdNqQ</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>CIDQCBAAAIAQKBQBAECQADABA4AA4AQBAAOSGAQCAYLCQAQCAADAUBIBAIDD4AICAAEQCBAAAMAQMBQ5AEDAAMAA</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Bilgewater|Demacia</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04DE002","n":3},{"c":"05BW001","n":3},{"c":"05DE012","n":3},{"c":"07DE014","n":3},{"c":"01DE029","n":3},{"c":"01DE035","n":3},{"c":"02BW022","n":3},{"c":"02BW040","n":3},{"c":"02DE006","n":3},{"c":"02DE010","n":3},{"c":"02BW062","n":2},{"c":"02DE009","n":2},{"c":"04DE003","n":2},{"c":"06BW029","n":2},{"c":"06DE048","n":2}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Keldog</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1CKHt5W262OqVUahdjh11tOI_iLOClJy8SS9v3HT9RIEWsSJ40CQAUPI_xtuajXdOFC7cdvA3xsd3A</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>CQCQCBACBYAQMAQJAEDAKDYBBECQ2AQBAUKROBIBAEBASAIHAUBACCAFFEBACBIEFIBAMBIMFYBQCCIKCQBQMBIHBYIAIAIFAEBQ6HI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Ionia|Mount Targon|Noxus|Shadow Isles|Shurima</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04IO014","n":3},{"c":"06IO009","n":3},{"c":"06SI015","n":3},{"c":"09SI013","n":3},{"c":"01SI021","n":3},{"c":"01SI023","n":3},{"c":"01IO009","n":2},{"c":"07SI002","n":2},{"c":"08SI041","n":2},{"c":"01SI004","n":2},{"c":"01SI042","n":2},{"c":"06SI012","n":2},{"c":"06SI046","n":2},{"c":"01MT010","n":1},{"c":"20NX006","n":1},{"c":"05SH014","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Borden</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>317</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>qK9glayGZ5epQctvwehXPI9r5oRK7o06vZ6d6XJXNy_B35V-NIfKnsbD6sbg9oW4vlzESUqjtMEecA</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>CECACBIEAYAQQAITAEEAIGADAECAQGJ2AYAQCBBUAEBQCAQBAQAQUAIIAEMAEAIBAEPAIBIEAIFA4GIBAIAQCFRK</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Freljord|Piltover &amp; Zaun</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>aggro</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"05PZ006","n":3},{"c":"08FR019","n":3},{"c":"08PZ024","n":3},{"c":"01PZ008","n":3},{"c":"01PZ025","n":3},{"c":"01PZ058","n":3},{"c":"01PZ052","n":2},{"c":"03FR002","n":2},{"c":"04FR010","n":2},{"c":"08FR024","n":2},{"c":"01FR001","n":2},{"c":"01FR030","n":2},{"c":"05PZ002","n":2},{"c":"05PZ010","n":2},{"c":"05PZ014","n":2},{"c":"05PZ025","n":2},{"c":"02FR001","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>mbrookz</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>iMQDykjthqoztGrFSrHwtphL2pV9BIrGgAz1EIFDSRHTboYbSYy9SPFPyLCvPzq3i5PdNMVJIeWEiA</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>CIEQCAIADUAQEAAGAECAAAYBAUAAYAIGAYOQCBQEBAAQOAAFAEEAABQEAYAAMCQVDQBACAIABIAQMABAAA</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Bilgewater|Demacia|Piltover &amp; Zaun</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01DE029","n":3},{"c":"02DE006","n":3},{"c":"04DE003","n":3},{"c":"05DE012","n":3},{"c":"06BW029","n":3},{"c":"06PZ008","n":3},{"c":"07DE005","n":3},{"c":"08DE006","n":3},{"c":"06DE006","n":3},{"c":"06DE010","n":3},{"c":"06DE021","n":3},{"c":"06DE028","n":3},{"c":"01DE010","n":2},{"c":"06DE032","n":2}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Mzhkm</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>wKRwXzXitOo8tiys3ThWEcY6NOqbxCgRL6LZa2_S69LCgiqhZdeCqkDtBim83OCOSHJ0lI82rvz5uA</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>CQDQCAICFEAQCBBUAEBQEFABAMCAWAIGAQJACBYCBMAQSAR2A4AQCARRAEBAEBIBAUCBSAIGAQVACCAKAYAQQAQKAIDQEEIUAMAQKBBGAEDAEIABA4BAS</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|F32|Freljord|Ionia|Piltover &amp; Zaun|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01IO041","n":3},{"c":"01PZ052","n":3},{"c":"03IO020","n":3},{"c":"03PZ011","n":3},{"c":"06PZ018","n":3},{"c":"07IO011","n":3},{"c":"09IO058","n":3},{"c":"01IO049","n":2},{"c":"02IO005","n":2},{"c":"05PZ025","n":2},{"c":"06PZ042","n":2},{"c":"08BC006","n":2},{"c":"08IO010","n":2},{"c":"07IO017","n":2},{"c":"07IO020","n":2},{"c":"01SI004","n":1},{"c":"38FR006","n":1},{"c":"02F32001","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>hungrylouna129</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4DksskDtcvxtt8JMYwyNMjIIbmau_tz4KwUT-zwcbizxUo3ZMm990UGyxvJ8PHKAEDre0lfPtNGyMw</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>CECQCAIFGEAQQAY4AMCAKBBWG4BQQBIHFEVAKBQFCQNSAJZOAAAQCBQFFU</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Bilgewater|Noxus|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01SI049","n":3},{"c":"08NX028","n":3},{"c":"04SI004","n":3},{"c":"04SI054","n":3},{"c":"04SI055","n":3},{"c":"08SI007","n":3},{"c":"08SI041","n":3},{"c":"08SI042","n":3},{"c":"06SI020","n":3},{"c":"06SI027","n":3},{"c":"06SI032","n":3},{"c":"06SI039","n":3},{"c":"06SI046","n":3},{"c":"01BW005","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>NotreDammit</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Ik2qUvSnwi86IeXEu5fiNj4mTgE6LR2fHlKi_J1gS05olorTm2il2QpyaTh-gdM17lDLdfXLjcZ3lw</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>CQBQCBAFGYAQMBIUAIEAKBZJAYAQSCQUAEEQKDICAECQCMICAYCSKLQCBACSKKQEAQCQIBJVG4CACBAFHAAQKCT7AEDAKJYBA4CQU</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|F127|Freljord|Piltover &amp; Zaun|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04SI054","n":3},{"c":"06SI020","n":3},{"c":"08SI007","n":3},{"c":"08SI041","n":3},{"c":"09BC020","n":2},{"c":"09SI013","n":2},{"c":"01SI001","n":2},{"c":"01SI049","n":2},{"c":"06SI037","n":2},{"c":"06SI046","n":2},{"c":"08SI037","n":2},{"c":"08SI042","n":2},{"c":"04SI004","n":2},{"c":"04SI005","n":2},{"c":"04SI053","n":2},{"c":"04SI055","n":2},{"c":"01PZ005","n":1},{"c":"56FR005","n":1},{"c":"10F127001","n":1},{"c":"06SI039","n":1}]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Resultados de la reducción de dimensionalidad
</commit_message>
<xml_diff>
--- a/lor_dataset.xlsx
+++ b/lor_dataset.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1772,16 +1772,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>2</v>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Borden</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
-        <v>317</v>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>317.0</t>
+        </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -1798,20 +1802,30 @@
           <t>Freljord|Piltover &amp; Zaun</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="K24" s="2" t="n">
-        <v>43.6</v>
-      </c>
-      <c r="L24" s="2" t="n">
-        <v>5.1</v>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>51.3</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>43.6</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
@@ -1830,16 +1844,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
-        <v>5</v>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>mbrookz</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n">
-        <v>237</v>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>237.0</t>
+        </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -1856,11 +1874,15 @@
           <t>Bilgewater|Demacia|Piltover &amp; Zaun</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I25" s="2" t="n">
-        <v>14</v>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
@@ -1878,16 +1900,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
-        <v>8</v>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Mzhkm</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
-        <v>198</v>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>198.0</t>
+        </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -1904,11 +1930,15 @@
           <t>Bandle City|F32|Freljord|Ionia|Piltover &amp; Zaun|Shadow Isles</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>18</v>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
@@ -1926,16 +1956,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
-        <v>12</v>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>hungrylouna129</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n">
-        <v>160</v>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>160.0</t>
+        </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -1952,11 +1986,15 @@
           <t>Bilgewater|Noxus|Shadow Isles</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I27" s="2" t="n">
-        <v>14</v>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
@@ -1974,16 +2012,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
-        <v>14</v>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>NotreDammit</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n">
-        <v>146</v>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>146.0</t>
+        </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -2000,11 +2042,15 @@
           <t>Bandle City|F127|Freljord|Piltover &amp; Zaun|Shadow Isles</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I28" s="2" t="n">
-        <v>20</v>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
@@ -2016,6 +2062,198 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Evilkyatt</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>VIhWFnBFEMr4EV5Wso7qWAXeLXjX7AsH9jGXBsQMzElxqWDkmhYduySwqjiw2LKgm8Vl4x7vCePEVA</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>CIEACAIEFUAQKAAMAEDAMHIBA4AAKAIIAAFACCAJAMBAMAAVDQBAMBAIEYBQCAQAAIAQIAADAIDAABQKAIAQKBBGAEDAAGA</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Bilgewater|Demacia|Freljord|Mount Targon|Piltover &amp; Zaun|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01PZ045","n":3},{"c":"05DE012","n":3},{"c":"06BW029","n":3},{"c":"07DE005","n":3},{"c":"08DE010","n":3},{"c":"08MT003","n":3},{"c":"06DE021","n":3},{"c":"06DE028","n":3},{"c":"06PZ008","n":3},{"c":"06PZ038","n":3},{"c":"02DE002","n":2},{"c":"04DE003","n":2},{"c":"06DE006","n":2},{"c":"06DE010","n":2},{"c":"01SI004","n":1},{"c":"38FR006","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Im Bard Out</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Yz3vZckMMsL-Dws1t-3XJfGXMMs6-aF_NVmV38P_BTavVKVSeopCEa87wrihIzczQX0FLehUySyTFw</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>CUCQCAYECMAQMCRLAEDQYDYBBEAQUAQBAEEBABQBAEBSEAIBAQKACAQBAMAQQBAZAEEQODACAQDTCOYIAEAQAMIBAEASWAIBAICQCAIFEUAQEBQKAEBQSJYBAQAQ6AIGAEKQ</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|F43|Freljord|Ionia|Mount Targon|Noxus|Piltover &amp; Zaun|Runeterra|Shurima</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"03PZ019","n":3},{"c":"06BC043","n":3},{"c":"07RU015","n":3},{"c":"09FR010","n":3},{"c":"01FR008","n":3},{"c":"01FR016","n":3},{"c":"01NX034","n":2},{"c":"01PZ020","n":2},{"c":"02FR003","n":2},{"c":"08PZ025","n":2},{"c":"09SH012","n":2},{"c":"04SH049","n":2},{"c":"04SH059","n":2},{"c":"01FR000","n":1},{"c":"49FR001","n":1},{"c":"01F43001","n":1},{"c":"01IO005","n":1},{"c":"01FR005","n":1},{"c":"37FR002","n":1},{"c":"06BC001","n":1},{"c":"03MT039","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>waitimplaying</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>_azDPaOzvLiVWYOIu_tqeRsKBR8jGB0PqWIwKWT4Q7tkGYQL315DorDP9xtQYmJXyLKmpxH_bxvxjA</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>CECQCBAABAAQMARDAEDQABICAEBCAKYDAEAASGQ5AUAQEAABAEBQADQBAQAAEAIGAAYACCAAAYCQCAYAAYAQGAQJAEDAEJQBBAAAUAQBAISTC</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Demacia|F08|Freljord|Ionia|Mount Targon|Noxus</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04DE008","n":3},{"c":"06IO035","n":3},{"c":"07DE005","n":3},{"c":"01IO032","n":3},{"c":"01IO043","n":3},{"c":"01DE009","n":3},{"c":"01DE026","n":3},{"c":"01DE029","n":3},{"c":"02DE001","n":2},{"c":"03DE014","n":2},{"c":"04DE002","n":2},{"c":"06DE048","n":2},{"c":"08DE006","n":2},{"c":"01NX000","n":1},{"c":"06FR003","n":1},{"c":"02MT001","n":1},{"c":"06IO038","n":1},{"c":"01F08000","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>iNilesD</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>wyBqeP-e5g-DWGj1HtegH7itQvt6v4ICyf548MkkPS2eOQAg1oZuz0NOBM3NpzMY4X3b_j_0lyxQ8g</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>CMDQCAIEGQAQGBADAECQOFQBAYDTAAIIAQEQEBAEAIDQIBAHE4WU63IDAEDQICIBBABQYAIIAQEACAIIAQBA</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>F08|Noxus|Piltover &amp; Zaun|Shurima</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"01PZ052","n":3},{"c":"03PZ003","n":3},{"c":"05SH022","n":3},{"c":"06SH048","n":3},{"c":"08PZ009","n":3},{"c":"04PZ002","n":3},{"c":"04PZ007","n":3},{"c":"04SH039","n":3},{"c":"04SH045","n":3},{"c":"04SH079","n":3},{"c":"04SH109","n":3},{"c":"07PZ009","n":2},{"c":"08NX012","n":2},{"c":"08PZ008","n":2},{"c":"01F08004","n":1}]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización de la API key
</commit_message>
<xml_diff>
--- a/lor_dataset.xlsx
+++ b/lor_dataset.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2068,16 +2068,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
-        <v>16</v>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Evilkyatt</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n">
-        <v>141</v>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>141.0</t>
+        </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -2094,11 +2098,15 @@
           <t>Bilgewater|Demacia|Freljord|Mount Targon|Piltover &amp; Zaun|Shadow Isles</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I29" s="2" t="n">
-        <v>16</v>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
@@ -2116,16 +2124,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
-        <v>18</v>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Im Bard Out</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n">
-        <v>135</v>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>135.0</t>
+        </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -2142,11 +2154,15 @@
           <t>Bandle City|F43|Freljord|Ionia|Mount Targon|Noxus|Piltover &amp; Zaun|Runeterra|Shurima</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>21</v>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
@@ -2164,16 +2180,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
-        <v>24</v>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
           <t>waitimplaying</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n">
-        <v>124</v>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>124.0</t>
+        </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
@@ -2190,11 +2210,15 @@
           <t>Demacia|F08|Freljord|Ionia|Mount Targon|Noxus</t>
         </is>
       </c>
-      <c r="H31" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I31" s="2" t="n">
-        <v>18</v>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
@@ -2212,16 +2236,20 @@
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
-        <v>29</v>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
           <t>iNilesD</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
-        <v>100</v>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -2238,11 +2266,15 @@
           <t>F08|Noxus|Piltover &amp; Zaun|Shurima</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I32" s="2" t="n">
-        <v>15</v>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
@@ -2254,6 +2286,256 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>DrChekhov42</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>1c4nwBwSyv5F1x83lL5dfhKFmmilYJSGA5t0If7XkaoDeMUcqouHaokbFO8-2k5ClT0A1DDCqeWjkw</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>CQDACBQFEAAQOBICAEEAABQBBECQ4AQJBIARIAYBAEFREJQCAIAQKAIDAQAQCAIHDYVACAIBAUOQ</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|Demacia|Freljord|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"06SI032","n":3},{"c":"07SI002","n":3},{"c":"08DE006","n":3},{"c":"09SI014","n":3},{"c":"09BC001","n":3},{"c":"09BC020","n":3},{"c":"01FR011","n":3},{"c":"01FR018","n":3},{"c":"01FR038","n":3},{"c":"01SI001","n":2},{"c":"01SI003","n":2},{"c":"01FR001","n":2},{"c":"01FR007","n":2},{"c":"01FR030","n":2},{"c":"01FR042","n":2},{"c":"01FR005","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Carrot Spirit</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>NF9ZwowvSyBz45YcetDzIlsyVLSXCW7enL4zTVyKjr2XKr2XBFWy1fc_CdtXAjFtiOBxXQRJAYTRUA</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>CQDACAQDAMAQMCQ2AEDAGKIBBEFAWBABAMBAYKBXAQCQUBZJUMA2MAICAEAQGGIBAUFHIAA</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Bandle City|Noxus</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"02NX003","n":3},{"c":"06BC026","n":3},{"c":"06NX041","n":3},{"c":"09BC011","n":3},{"c":"01NX002","n":3},{"c":"01NX012","n":3},{"c":"01NX040","n":3},{"c":"01NX055","n":3},{"c":"05BC007","n":3},{"c":"05BC041","n":3},{"c":"05BC163","n":3},{"c":"05BC166","n":3},{"c":"01NX025","n":2},{"c":"05BC116","n":2}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Davebo</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>VLKpCAmlUM3NEPhfXqQhNpavrwVpFqBTl0XhrDvMARySiqz6PJyEtbCAExJgF-KsxVkqbVZgpxDFSQ</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>CEDACBYECEAQQAITAEEAIGACAEAQIHQDAUCAEBQOAQAQICAZGQ5ACAIBAEVAEAIBAEAQCBABBI</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Freljord|Piltover &amp; Zaun</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>midrange</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"07PZ017","n":3},{"c":"08FR019","n":3},{"c":"08PZ024","n":3},{"c":"01FR004","n":3},{"c":"01FR030","n":3},{"c":"05PZ002","n":3},{"c":"05PZ006","n":3},{"c":"05PZ014","n":3},{"c":"01PZ008","n":3},{"c":"01PZ025","n":3},{"c":"01PZ052","n":3},{"c":"01PZ058","n":3},{"c":"01FR042","n":2},{"c":"01FR001","n":1},{"c":"01FR004","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Scilla</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>vwIBeem3KeMHt2DXT689hGEUoZwydZ1S7q2GcWLHvl4GxNDmaxHhI4X25Rx9afLQ0Z4io5Xm3dC2-A</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>CEAAAAICAAAAMJY</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Demacia</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"02DE000","n":1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Keldog</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>1CKHt5W262OqVUahdjh11tOI_iLOClJy8SS9v3HT9RIEWsSJ40CQAUPI_xtuajXdOFC7cdvA3xsd3A</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>CQCQCBACBYAQMAQJAEDAKDYBBECQ2AQBAUKROBIBAEBASAIHAUBACCAFFEBAMBIMFYBQCBIBAQVAGAIJBIKAEAIFAMOQGBQFA4HBA</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Ionia|Mount Targon|Noxus|Shadow Isles</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>[{"c":"04IO014","n":3},{"c":"06IO009","n":3},{"c":"06SI015","n":3},{"c":"09SI013","n":3},{"c":"01SI021","n":3},{"c":"01SI023","n":3},{"c":"01IO009","n":2},{"c":"07SI002","n":2},{"c":"08SI041","n":2},{"c":"06SI012","n":2},{"c":"06SI046","n":2},{"c":"01SI001","n":2},{"c":"01SI004","n":2},{"c":"01SI042","n":2},{"c":"01MT010","n":1},{"c":"20IO001","n":1},{"c":"05NX029","n":1}]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>